<commit_message>
Refactor eCitizen module; add reconciliation
Rework the eCitizen module: remove custom logger/components and ActiveRecord models; add a dedicated SMIS DB connection (from modules/ecitizen/.env) and stricter HostControl. PaymentService rewritten to use direct SQL, introduce reconciliation (reconcile-settled), new reconciliation statuses, and payment-status querying (statusUrl, caBundlePath support). UI: hide legacy "Complete payment" button and support a configured bankAccountId. Config updates in credentials/module and new operational docs (ECITIZEN_PAYMENT_CONFIRMATION_AND_RECONCILIATION.md). Note: module now throws if SMIS .env is missing and requires allowed hosts/configured URLs.
</commit_message>
<xml_diff>
--- a/modules/ecitizen/NDU SERVICE CODES.xlsx
+++ b/modules/ecitizen/NDU SERVICE CODES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\odhis\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{245C18B9-80F3-459D-BAC9-8F19BB2DBCE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF16018E-9508-4CCA-831D-20CEF099B777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>Diploma Graduation Package.</t>
   </si>
@@ -75,6 +75,9 @@
     <t>Certificate Correction</t>
   </si>
   <si>
+    <t>Transcripts/Certificates Verification &amp;Certification</t>
+  </si>
+  <si>
     <t>Replacement of Lost Damaged or Stolen Transcripts</t>
   </si>
   <si>
@@ -90,23 +93,47 @@
     <t>Student Reinstatement (Overstay)</t>
   </si>
   <si>
+    <t>Masters Tuition Fee 2025/2026 Sem 1</t>
+  </si>
+  <si>
+    <t>PhD Tuition Fee 2025/2026 Sem 1</t>
+  </si>
+  <si>
+    <t>PhD in Crisis Response and Disaster&amp;nbsp;Management</t>
+  </si>
+  <si>
+    <t>Masters of Arts in Gender and Peace Support Studies</t>
+  </si>
+  <si>
+    <t>Semester 1 Fees</t>
+  </si>
+  <si>
+    <t>Supplementary Exam Application</t>
+  </si>
+  <si>
+    <t>Semester 4 Fees</t>
+  </si>
+  <si>
+    <t>Semester 3 Fees</t>
+  </si>
+  <si>
+    <t>Semester 2 Fees</t>
+  </si>
+  <si>
+    <t>Master of Arts in Crisis Response and Disaster Management</t>
+  </si>
+  <si>
     <t xml:space="preserve">SERVICE </t>
   </si>
   <si>
     <t>SERVICE CODE</t>
-  </si>
-  <si>
-    <t>Transcripts/Certificates Verification &amp;Cedification</t>
-  </si>
-  <si>
-    <t>Tuition and Related Fees</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -133,13 +160,6 @@
       <color rgb="FF00D97E"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -183,7 +203,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -194,7 +214,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -475,23 +494,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <dimension ref="A1:H33"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="44.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.7109375" style="1"/>
+    <col min="1" max="1" width="44.54296875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="5" customFormat="1">
+    <row r="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -505,7 +524,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -519,7 +538,7 @@
       <c r="G3" s="2"/>
       <c r="H3" s="3"/>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -533,7 +552,7 @@
       <c r="G4" s="2"/>
       <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -547,7 +566,7 @@
       <c r="G5" s="2"/>
       <c r="H5" s="3"/>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -561,7 +580,7 @@
       <c r="G6" s="2"/>
       <c r="H6" s="3"/>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -575,7 +594,7 @@
       <c r="G7" s="2"/>
       <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -589,7 +608,7 @@
       <c r="G8" s="2"/>
       <c r="H8" s="3"/>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -603,7 +622,7 @@
       <c r="G9" s="2"/>
       <c r="H9" s="3"/>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -617,7 +636,7 @@
       <c r="G10" s="2"/>
       <c r="H10" s="3"/>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -631,7 +650,7 @@
       <c r="G11" s="2"/>
       <c r="H11" s="3"/>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -645,7 +664,7 @@
       <c r="G12" s="2"/>
       <c r="H12" s="3"/>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -659,7 +678,7 @@
       <c r="G13" s="2"/>
       <c r="H13" s="3"/>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -673,7 +692,7 @@
       <c r="G14" s="2"/>
       <c r="H14" s="3"/>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -687,7 +706,7 @@
       <c r="G15" s="2"/>
       <c r="H15" s="3"/>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -701,7 +720,7 @@
       <c r="G16" s="2"/>
       <c r="H16" s="3"/>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
@@ -715,9 +734,9 @@
       <c r="G17" s="2"/>
       <c r="H17" s="3"/>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B18" s="2">
         <v>15247531</v>
@@ -729,9 +748,9 @@
       <c r="G18" s="2"/>
       <c r="H18" s="3"/>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B19" s="2">
         <v>15247530</v>
@@ -743,9 +762,9 @@
       <c r="G19" s="2"/>
       <c r="H19" s="3"/>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B20" s="2">
         <v>15247529</v>
@@ -757,9 +776,9 @@
       <c r="G20" s="2"/>
       <c r="H20" s="3"/>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B21" s="2">
         <v>15247528</v>
@@ -771,9 +790,9 @@
       <c r="G21" s="2"/>
       <c r="H21" s="3"/>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B22" s="2">
         <v>15247527</v>
@@ -785,11 +804,11 @@
       <c r="G22" s="2"/>
       <c r="H22" s="3"/>
     </row>
-    <row r="23" spans="1:8" ht="15.75">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B23" s="6">
+        <v>21</v>
+      </c>
+      <c r="B23" s="2">
         <v>15247526</v>
       </c>
       <c r="C23" s="2"/>
@@ -799,9 +818,9 @@
       <c r="G23" s="2"/>
       <c r="H23" s="3"/>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B24" s="2">
         <v>15245097</v>
@@ -813,9 +832,13 @@
       <c r="G24" s="2"/>
       <c r="H24" s="3"/>
     </row>
-    <row r="25" spans="1:8">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" s="2">
+        <v>15245096</v>
+      </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
@@ -823,15 +846,117 @@
       <c r="G25" s="2"/>
       <c r="H25" s="3"/>
     </row>
-    <row r="26" spans="1:8">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="2">
+        <v>15240693</v>
+      </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="3"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" s="2">
+        <v>15240692</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="3"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" s="2">
+        <v>15239274</v>
+      </c>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="3"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" s="2">
+        <v>15239273</v>
+      </c>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="3"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="2">
+        <v>15239272</v>
+      </c>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="3"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" s="2">
+        <v>15239271</v>
+      </c>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="3"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32" s="2">
+        <v>15239270</v>
+      </c>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="3"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" s="2">
+        <v>15239269</v>
+      </c>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>